<commit_message>
fix(data): correct ENEM spreadsheet entries with missing answers and incorrect statements
</commit_message>
<xml_diff>
--- a/data/ENEM --- Conhecimento do ENEM de 2020 à 2025.xlsx
+++ b/data/ENEM --- Conhecimento do ENEM de 2020 à 2025.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1575" uniqueCount="1575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1571" uniqueCount="1571">
   <si>
     <t>question</t>
   </si>
@@ -1365,12 +1365,6 @@
     <t>B - Salto em altura.</t>
   </si>
   <si>
-    <t>ENEM 2024 - Ciências da Natureza - QUESTÃO 111 O exoesqueleto dos crustáceos é formado por quitina e impregnações de sais calcários e, por isso, é mais duro quando comparado com o exoesqueleto de outros artrópodes. Esse revestimento externo confere proteção, mas, por ser duro, limita o crescimento desses animais. C Para superar essa limitação, o exoesqueleto deve ser A formado somente na fase adulta do animal. B fragmentado para expansão nas áreas de articulação. C modelado continuamente para ajuste ao tamanho do corpo. D substituído por meio de mudas que ocorrem periodicamente. D E impregnado por pequena quantidade de sais para sua distensão. E</t>
-  </si>
-  <si>
-    <t>D - texto da alternativa não disponível na planilha</t>
-  </si>
-  <si>
     <t>ENEM 2024 - Ciências da Natureza - QUESTÃO 112 O Cerrado e a Amazônia abrigam grande número de Um dos exemplos mais conhecidos de herança serpentes popularmente conhecidas como cobras-corais. recessiva ligada ao cromossomo X é o daltonismo. Na Amazônia predominam as corais-verdadeiras, que Como em qualquer distúrbio recessivo ligado ao são peçonhentas, enquanto no Cerrado prevalecem as cromossomo X, existem muito mais homens apresentando falsas-corais, que não possuem peçonha. Essas espécies o fenótipo com esse tipo de daltonismo do que mulheres. apresentam um padrão de coloração muito semelhante. Um casal formado por um homem não daltônico e por uma Essa similaridade traz uma vantagem tanto para as corais mulher gestante também não daltônica, mas portadora falsas como para as verdadeiras. do gene recessivo para esse tipo de daltonismo, está esperando um bebê. Em uma das consultas de pré-natal, FRANÇA, F. G. R. [...] serpentes corais em ambientes campestres, savânicos e florestais da América do Sul. o casal recebeu um heredograma que contém todas as Brasília: UnB, 2008 (adaptado). possibilidades de genótipo para esse bebê. Considere a legenda: Nas fotografias, são apresentados exemplos dessas serpentes: uma coral-verdadeira e uma falsa-coral. Mulher heterozigota portadora do gene para daltonismo Mulher não daltônica Mulher daltônica Homem não daltônico Homem daltônico GRIFFITHS, A. et al. Introdução à genética. Rio de Janeiro: SILVA, L. C.; COTTA, G. A.; RESENDE, F. C. Cobra-coral: aplicativo Guanabara Koogan, 2016 (adaptado). educativo para reconhecimento das cobras-corais do estado de Minas Gerais, Brasil. Herpetologia Brasileira, Qual heredograma foi recebido pelo casal? n. 1, 2021 (adaptado). Qual é a vantagem dessa similaridade para as falsas-corais? A A Facilita a captura de presas. B Diminui a competição por recursos. C Possibilita a geração de indivíduos híbridos. D Reduz a possibilidade de sofrerem predação. E Otimiza o encontro de parceiros reprodutivos. B</t>
   </si>
   <si>
@@ -3436,12 +3430,6 @@
   </si>
   <si>
     <t>E - obter moléculas de cDNA viral por meio da transcrição reversa.</t>
-  </si>
-  <si>
-    <t>ENEM 2022 - Ciências da Natureza - QUESTÃO 128 8 O quadro mostra valores de corrente elétrica e seus efeitos sobre o corpo humano. Corrente elétrica Dano físico Até 10 mA Dor e contração muscular De 10 mA até 20 mA Aumento das contrações musculares De 20 mA até 100 mA Parada respiratória De 100 mA até 3 A Fibrilação ventricular Acima de 3 A Parada cardíaca e queimaduras A corrente elétrica que percorrerá o corpo de um indivíduo depende da tensão aplicada e da resistência elétrica média do corpo humano. Esse último fator está intimamente relacionado com a umidade da pele, que seca apresenta resistência elétrica da ordem de 500 kΩ, mas, se molhada, pode chegar a apenas 1 kΩ. Apesar de incomum, é possível sofrer um acidente utilizando baterias de 12 V. Considere que um indivíduo com a pele molhada sofreu uma parada respiratória ao tocar simultaneamente nos pontos A e B de uma associação de duas dessas baterias. DURAN, J. E. R. Biofísica: fundamentos e aplicações. São Paulo: Pearson Prentice Hall, 2003 (adaptado). Qual associação de baterias foi responsável pelo acidente? A - + A B - + B - + A B - + C A B - + - + D + A B - - + E A B - + - +</t>
-  </si>
-  <si>
-    <t>A - texto da alternativa não disponível na planilha</t>
   </si>
   <si>
     <t>ENEM 2022 - Ciências da Natureza - QUESTÃO 129 9 O urânio é empregado como fonte de energia em reatores nucleares. Para tanto, o seu mineral deve ser refinado, convertido a hexafluoreto de urânio e posteriormente enriquecido, para aumentar de 0,7% a 3% a abundância de um isótopo específico — o urânio-235. Uma das formas de enriquecimento utiliza a pequena diferença de massa entre os hexafluoretos de urânio-235 e de urânio-238 para separá-los por efusão, precedida pela vaporização. Esses vapores devem efundir repetidamente milhares de vezes através de barreiras porosas formadas por telas com grande número de pequenos orifícios. No entanto, devido à complexidade e à grande quantidade de energia envolvida, cientistas e engenheiros continuam a pesquisar procedimentos alternativos de enriquecimento. ATKINS, P.; JONES, L. Princípios de química: questionando a vida moderna e o meio ambiente. Porto Alegre: Bookman, 2006 (adaptado). Considerando a diferença de massa mencionada entre os dois isótopos, que tipo de procedimento alternativo ao da efusão pode ser empregado para tal finalidade? A A Peneiração. B B Centrifugação. C C Extração por solvente. D D Destilação fracionada. E E Separação magnética.</t>
@@ -4855,10 +4843,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;#xFF2D;&amp;#xFF33; &amp;#xFF30;&amp;#x30B4;&amp;#x30B7;&amp;#x30C3;&amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;#xB9D1;&amp;#xC740; &amp;#xACE0;&amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;#x5B8B;&amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;#x65B0;&amp;#x7D30;&amp;#x660E;&amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="&amp;amp;#xFF2D;&amp;amp;#xFF33; &amp;amp;#xFF30;&amp;amp;#x30B4;&amp;amp;#x30B7;&amp;amp;#x30C3;&amp;amp;#x30AF;"/>
+        <a:font script="Hang" typeface="&amp;amp;#xB9D1;&amp;amp;#xC740; &amp;amp;#xACE0;&amp;amp;#xB515;"/>
+        <a:font script="Hans" typeface="&amp;amp;#x5B8B;&amp;amp;#x4F53;"/>
+        <a:font script="Hant" typeface="&amp;amp;#x65B0;&amp;amp;#x7D30;&amp;amp;#x660E;&amp;amp;#x9AD4;"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -4889,10 +4877,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;#xFF2D;&amp;#xFF33; &amp;#xFF30;&amp;#x30B4;&amp;#x30B7;&amp;#x30C3;&amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;#xB9D1;&amp;#xC740; &amp;#xACE0;&amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;#x5B8B;&amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;#x65B0;&amp;#x7D30;&amp;#x660E;&amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="&amp;amp;#xFF2D;&amp;amp;#xFF33; &amp;amp;#xFF30;&amp;amp;#x30B4;&amp;amp;#x30B7;&amp;amp;#x30C3;&amp;amp;#x30AF;"/>
+        <a:font script="Hang" typeface="&amp;amp;#xB9D1;&amp;amp;#xC740; &amp;amp;#xACE0;&amp;amp;#xB515;"/>
+        <a:font script="Hans" typeface="&amp;amp;#x5B8B;&amp;amp;#x4F53;"/>
+        <a:font script="Hant" typeface="&amp;amp;#x65B0;&amp;amp;#x7D30;&amp;amp;#x660E;&amp;amp;#x9AD4;"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -5093,8 +5081,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{214B4059-A289-43DE-90AE-1D8F30E51581}" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:B796"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E5FC641B-E54E-4507-A1CB-C51837885EDF}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:B794"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="72.421875" customWidth="1"/>
@@ -7242,15 +7230,15 @@
         <v>534</v>
       </c>
       <c r="B268" t="s">
-        <v>535</v>
+        <v>321</v>
       </c>
     </row>
     <row r="269" ht="15" customHeight="1">
       <c r="A269" t="s">
+        <v>535</v>
+      </c>
+      <c r="B269" t="s">
         <v>536</v>
-      </c>
-      <c r="B269" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="270" ht="15" customHeight="1">
@@ -7590,18 +7578,18 @@
       </c>
     </row>
     <row r="312" ht="15" customHeight="1">
-      <c r="A312" t="s">
+      <c r="A312" s="1" t="s">
         <v>621</v>
       </c>
-      <c r="B312" t="s">
+      <c r="B312" s="1" t="s">
         <v>622</v>
       </c>
     </row>
     <row r="313" ht="15" customHeight="1">
-      <c r="A313" s="1" t="s">
+      <c r="A313" t="s">
         <v>623</v>
       </c>
-      <c r="B313" s="1" t="s">
+      <c r="B313" t="s">
         <v>624</v>
       </c>
     </row>
@@ -7649,7 +7637,7 @@
       <c r="A319" t="s">
         <v>635</v>
       </c>
-      <c r="B319" t="s">
+      <c r="B319" s="1" t="s">
         <v>636</v>
       </c>
     </row>
@@ -7657,7 +7645,7 @@
       <c r="A320" t="s">
         <v>637</v>
       </c>
-      <c r="B320" s="1" t="s">
+      <c r="B320" t="s">
         <v>638</v>
       </c>
     </row>
@@ -7745,7 +7733,7 @@
       <c r="A331" t="s">
         <v>659</v>
       </c>
-      <c r="B331" t="s">
+      <c r="B331" s="1" t="s">
         <v>660</v>
       </c>
     </row>
@@ -7753,7 +7741,7 @@
       <c r="A332" t="s">
         <v>661</v>
       </c>
-      <c r="B332" s="1" t="s">
+      <c r="B332" t="s">
         <v>662</v>
       </c>
     </row>
@@ -8026,15 +8014,15 @@
         <v>729</v>
       </c>
       <c r="B366" t="s">
-        <v>730</v>
+        <v>279</v>
       </c>
     </row>
     <row r="367" ht="15" customHeight="1">
       <c r="A367" t="s">
+        <v>730</v>
+      </c>
+      <c r="B367" t="s">
         <v>731</v>
-      </c>
-      <c r="B367" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="368" ht="15" customHeight="1">
@@ -8145,7 +8133,7 @@
       <c r="A381" t="s">
         <v>758</v>
       </c>
-      <c r="B381" t="s">
+      <c r="B381" s="1" t="s">
         <v>759</v>
       </c>
     </row>
@@ -8153,7 +8141,7 @@
       <c r="A382" t="s">
         <v>760</v>
       </c>
-      <c r="B382" s="1" t="s">
+      <c r="B382" t="s">
         <v>761</v>
       </c>
     </row>
@@ -8209,7 +8197,7 @@
       <c r="A389" t="s">
         <v>774</v>
       </c>
-      <c r="B389" t="s">
+      <c r="B389" s="1" t="s">
         <v>775</v>
       </c>
     </row>
@@ -8217,7 +8205,7 @@
       <c r="A390" t="s">
         <v>776</v>
       </c>
-      <c r="B390" s="1" t="s">
+      <c r="B390" t="s">
         <v>777</v>
       </c>
     </row>
@@ -8314,15 +8302,15 @@
         <v>800</v>
       </c>
       <c r="B402" t="s">
-        <v>801</v>
+        <v>223</v>
       </c>
     </row>
     <row r="403" ht="15" customHeight="1">
       <c r="A403" t="s">
+        <v>801</v>
+      </c>
+      <c r="B403" t="s">
         <v>802</v>
-      </c>
-      <c r="B403" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="404" ht="15" customHeight="1">
@@ -8361,7 +8349,7 @@
       <c r="A408" t="s">
         <v>811</v>
       </c>
-      <c r="B408" t="s">
+      <c r="B408" s="1" t="s">
         <v>812</v>
       </c>
     </row>
@@ -8369,7 +8357,7 @@
       <c r="A409" t="s">
         <v>813</v>
       </c>
-      <c r="B409" s="1" t="s">
+      <c r="B409" t="s">
         <v>814</v>
       </c>
     </row>
@@ -8430,18 +8418,18 @@
       </c>
     </row>
     <row r="417" ht="15" customHeight="1">
-      <c r="A417" t="s">
+      <c r="A417" s="1" t="s">
         <v>829</v>
       </c>
-      <c r="B417" t="s">
+      <c r="B417" s="1" t="s">
         <v>830</v>
       </c>
     </row>
     <row r="418" ht="15" customHeight="1">
-      <c r="A418" s="1" t="s">
+      <c r="A418" t="s">
         <v>831</v>
       </c>
-      <c r="B418" s="1" t="s">
+      <c r="B418" t="s">
         <v>832</v>
       </c>
     </row>
@@ -8490,15 +8478,15 @@
         <v>843</v>
       </c>
       <c r="B424" t="s">
-        <v>844</v>
+        <v>313</v>
       </c>
     </row>
     <row r="425" ht="15" customHeight="1">
       <c r="A425" t="s">
+        <v>844</v>
+      </c>
+      <c r="B425" t="s">
         <v>845</v>
-      </c>
-      <c r="B425" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="426" ht="15" customHeight="1">
@@ -8657,7 +8645,7 @@
       <c r="A445" t="s">
         <v>884</v>
       </c>
-      <c r="B445" t="s">
+      <c r="B445" s="1" t="s">
         <v>885</v>
       </c>
     </row>
@@ -8665,7 +8653,7 @@
       <c r="A446" t="s">
         <v>886</v>
       </c>
-      <c r="B446" s="1" t="s">
+      <c r="B446" t="s">
         <v>887</v>
       </c>
     </row>
@@ -8849,7 +8837,7 @@
       <c r="A469" t="s">
         <v>932</v>
       </c>
-      <c r="B469" t="s">
+      <c r="B469" s="1" t="s">
         <v>933</v>
       </c>
     </row>
@@ -8857,7 +8845,7 @@
       <c r="A470" t="s">
         <v>934</v>
       </c>
-      <c r="B470" s="1" t="s">
+      <c r="B470" t="s">
         <v>935</v>
       </c>
     </row>
@@ -8897,7 +8885,7 @@
       <c r="A475" t="s">
         <v>944</v>
       </c>
-      <c r="B475" t="s">
+      <c r="B475" s="1" t="s">
         <v>945</v>
       </c>
     </row>
@@ -8905,7 +8893,7 @@
       <c r="A476" t="s">
         <v>946</v>
       </c>
-      <c r="B476" s="1" t="s">
+      <c r="B476" t="s">
         <v>947</v>
       </c>
     </row>
@@ -9409,7 +9397,7 @@
       <c r="A539" t="s">
         <v>1072</v>
       </c>
-      <c r="B539" t="s">
+      <c r="B539" s="1" t="s">
         <v>1073</v>
       </c>
     </row>
@@ -9417,7 +9405,7 @@
       <c r="A540" t="s">
         <v>1074</v>
       </c>
-      <c r="B540" s="1" t="s">
+      <c r="B540" t="s">
         <v>1075</v>
       </c>
     </row>
@@ -9497,7 +9485,7 @@
       <c r="A550" t="s">
         <v>1094</v>
       </c>
-      <c r="B550" t="s">
+      <c r="B550" s="1" t="s">
         <v>1095</v>
       </c>
     </row>
@@ -9513,7 +9501,7 @@
       <c r="A552" t="s">
         <v>1098</v>
       </c>
-      <c r="B552" s="1" t="s">
+      <c r="B552" t="s">
         <v>1099</v>
       </c>
     </row>
@@ -9522,15 +9510,15 @@
         <v>1100</v>
       </c>
       <c r="B553" t="s">
-        <v>1101</v>
+        <v>223</v>
       </c>
     </row>
     <row r="554" ht="15" customHeight="1">
       <c r="A554" t="s">
+        <v>1101</v>
+      </c>
+      <c r="B554" t="s">
         <v>1102</v>
-      </c>
-      <c r="B554" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="555" ht="15" customHeight="1">
@@ -9673,7 +9661,7 @@
       <c r="A572" t="s">
         <v>1137</v>
       </c>
-      <c r="B572" t="s">
+      <c r="B572" s="1" t="s">
         <v>1138</v>
       </c>
     </row>
@@ -9681,7 +9669,7 @@
       <c r="A573" t="s">
         <v>1139</v>
       </c>
-      <c r="B573" s="1" t="s">
+      <c r="B573" t="s">
         <v>1140</v>
       </c>
     </row>
@@ -9689,7 +9677,7 @@
       <c r="A574" t="s">
         <v>1141</v>
       </c>
-      <c r="B574" t="s">
+      <c r="B574" s="1" t="s">
         <v>1142</v>
       </c>
     </row>
@@ -9705,7 +9693,7 @@
       <c r="A576" t="s">
         <v>1145</v>
       </c>
-      <c r="B576" s="1" t="s">
+      <c r="B576" t="s">
         <v>1146</v>
       </c>
     </row>
@@ -9754,23 +9742,23 @@
         <v>1157</v>
       </c>
       <c r="B582" t="s">
-        <v>1158</v>
+        <v>531</v>
       </c>
     </row>
     <row r="583" ht="15" customHeight="1">
       <c r="A583" t="s">
+        <v>1158</v>
+      </c>
+      <c r="B583" t="s">
         <v>1159</v>
       </c>
-      <c r="B583" t="s">
+    </row>
+    <row r="584" ht="15" customHeight="1">
+      <c r="A584" s="1" t="s">
         <v>1160</v>
       </c>
-    </row>
-    <row r="584" ht="15" customHeight="1">
-      <c r="A584" t="s">
+      <c r="B584" s="1" t="s">
         <v>1161</v>
-      </c>
-      <c r="B584" t="s">
-        <v>533</v>
       </c>
     </row>
     <row r="585" ht="15" customHeight="1">
@@ -9778,31 +9766,31 @@
         <v>1162</v>
       </c>
       <c r="B585" t="s">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="586" ht="15" customHeight="1">
+      <c r="A586" t="s">
         <v>1163</v>
       </c>
-    </row>
-    <row r="586" ht="15" customHeight="1">
-      <c r="A586" s="1" t="s">
-        <v>1164</v>
-      </c>
-      <c r="B586" s="1" t="s">
-        <v>1165</v>
+      <c r="B586" t="s">
+        <v>859</v>
       </c>
     </row>
     <row r="587" ht="15" customHeight="1">
       <c r="A587" t="s">
-        <v>1166</v>
+        <v>1164</v>
       </c>
       <c r="B587" t="s">
-        <v>1163</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="588" ht="15" customHeight="1">
       <c r="A588" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B588" t="s">
         <v>1167</v>
-      </c>
-      <c r="B588" t="s">
-        <v>861</v>
       </c>
     </row>
     <row r="589" ht="15" customHeight="1">
@@ -9818,23 +9806,23 @@
         <v>1170</v>
       </c>
       <c r="B590" t="s">
-        <v>1171</v>
+        <v>877</v>
       </c>
     </row>
     <row r="591" ht="15" customHeight="1">
       <c r="A591" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B591" t="s">
         <v>1172</v>
-      </c>
-      <c r="B591" t="s">
-        <v>1173</v>
       </c>
     </row>
     <row r="592" ht="15" customHeight="1">
       <c r="A592" t="s">
+        <v>1173</v>
+      </c>
+      <c r="B592" t="s">
         <v>1174</v>
-      </c>
-      <c r="B592" t="s">
-        <v>879</v>
       </c>
     </row>
     <row r="593" ht="15" customHeight="1">
@@ -9890,23 +9878,23 @@
         <v>1187</v>
       </c>
       <c r="B599" t="s">
-        <v>1188</v>
+        <v>279</v>
       </c>
     </row>
     <row r="600" ht="15" customHeight="1">
       <c r="A600" t="s">
+        <v>1188</v>
+      </c>
+      <c r="B600" t="s">
         <v>1189</v>
-      </c>
-      <c r="B600" t="s">
-        <v>1190</v>
       </c>
     </row>
     <row r="601" ht="15" customHeight="1">
       <c r="A601" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B601" t="s">
         <v>1191</v>
-      </c>
-      <c r="B601" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="602" ht="15" customHeight="1">
@@ -9926,10 +9914,10 @@
       </c>
     </row>
     <row r="604" ht="15" customHeight="1">
-      <c r="A604" t="s">
+      <c r="A604" s="1" t="s">
         <v>1196</v>
       </c>
-      <c r="B604" t="s">
+      <c r="B604" s="1" t="s">
         <v>1197</v>
       </c>
     </row>
@@ -9942,10 +9930,10 @@
       </c>
     </row>
     <row r="606" ht="15" customHeight="1">
-      <c r="A606" s="1" t="s">
+      <c r="A606" t="s">
         <v>1200</v>
       </c>
-      <c r="B606" s="1" t="s">
+      <c r="B606" t="s">
         <v>1201</v>
       </c>
     </row>
@@ -10030,10 +10018,10 @@
       </c>
     </row>
     <row r="617" ht="15" customHeight="1">
-      <c r="A617" t="s">
+      <c r="A617" s="1" t="s">
         <v>1222</v>
       </c>
-      <c r="B617" t="s">
+      <c r="B617" s="1" t="s">
         <v>1223</v>
       </c>
     </row>
@@ -10042,23 +10030,23 @@
         <v>1224</v>
       </c>
       <c r="B618" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="619" ht="15" customHeight="1">
+      <c r="A619" t="s">
         <v>1225</v>
       </c>
-    </row>
-    <row r="619" ht="15" customHeight="1">
-      <c r="A619" s="1" t="s">
+      <c r="B619" t="s">
         <v>1226</v>
-      </c>
-      <c r="B619" s="1" t="s">
-        <v>1227</v>
       </c>
     </row>
     <row r="620" ht="15" customHeight="1">
       <c r="A620" t="s">
+        <v>1227</v>
+      </c>
+      <c r="B620" t="s">
         <v>1228</v>
-      </c>
-      <c r="B620" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="621" ht="15" customHeight="1">
@@ -10865,7 +10853,7 @@
       <c r="A721" t="s">
         <v>1429</v>
       </c>
-      <c r="B721" t="s">
+      <c r="B721" s="1" t="s">
         <v>1430</v>
       </c>
     </row>
@@ -10881,7 +10869,7 @@
       <c r="A723" t="s">
         <v>1433</v>
       </c>
-      <c r="B723" s="1" t="s">
+      <c r="B723" t="s">
         <v>1434</v>
       </c>
     </row>
@@ -10906,23 +10894,23 @@
         <v>1439</v>
       </c>
       <c r="B726" t="s">
-        <v>1440</v>
+        <v>789</v>
       </c>
     </row>
     <row r="727" ht="15" customHeight="1">
       <c r="A727" t="s">
+        <v>1440</v>
+      </c>
+      <c r="B727" t="s">
         <v>1441</v>
-      </c>
-      <c r="B727" t="s">
-        <v>1442</v>
       </c>
     </row>
     <row r="728" ht="15" customHeight="1">
       <c r="A728" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B728" t="s">
         <v>1443</v>
-      </c>
-      <c r="B728" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="729" ht="15" customHeight="1">
@@ -10953,7 +10941,7 @@
       <c r="A732" t="s">
         <v>1450</v>
       </c>
-      <c r="B732" t="s">
+      <c r="B732" s="1" t="s">
         <v>1451</v>
       </c>
     </row>
@@ -10962,23 +10950,23 @@
         <v>1452</v>
       </c>
       <c r="B733" t="s">
-        <v>1453</v>
+        <v>789</v>
       </c>
     </row>
     <row r="734" ht="15" customHeight="1">
       <c r="A734" t="s">
+        <v>1453</v>
+      </c>
+      <c r="B734" t="s">
         <v>1454</v>
-      </c>
-      <c r="B734" s="1" t="s">
-        <v>1455</v>
       </c>
     </row>
     <row r="735" ht="15" customHeight="1">
       <c r="A735" t="s">
+        <v>1455</v>
+      </c>
+      <c r="B735" t="s">
         <v>1456</v>
-      </c>
-      <c r="B735" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="736" ht="15" customHeight="1">
@@ -11089,7 +11077,7 @@
       <c r="A749" t="s">
         <v>1483</v>
       </c>
-      <c r="B749" t="s">
+      <c r="B749" s="1" t="s">
         <v>1484</v>
       </c>
     </row>
@@ -11105,7 +11093,7 @@
       <c r="A751" t="s">
         <v>1487</v>
       </c>
-      <c r="B751" s="1" t="s">
+      <c r="B751" t="s">
         <v>1488</v>
       </c>
     </row>
@@ -11162,31 +11150,31 @@
         <v>1501</v>
       </c>
       <c r="B758" t="s">
-        <v>1502</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="759" ht="15" customHeight="1">
       <c r="A759" t="s">
-        <v>1503</v>
+        <v>1502</v>
       </c>
       <c r="B759" t="s">
-        <v>1504</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="760" ht="15" customHeight="1">
       <c r="A760" t="s">
-        <v>1505</v>
+        <v>1503</v>
       </c>
       <c r="B760" t="s">
-        <v>1195</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="761" ht="15" customHeight="1">
       <c r="A761" t="s">
+        <v>1505</v>
+      </c>
+      <c r="B761" t="s">
         <v>1506</v>
-      </c>
-      <c r="B761" t="s">
-        <v>1504</v>
       </c>
     </row>
     <row r="762" ht="15" customHeight="1">
@@ -11290,23 +11278,23 @@
         <v>1531</v>
       </c>
       <c r="B774" t="s">
-        <v>1532</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="775" ht="15" customHeight="1">
       <c r="A775" t="s">
+        <v>1532</v>
+      </c>
+      <c r="B775" t="s">
         <v>1533</v>
-      </c>
-      <c r="B775" t="s">
-        <v>1534</v>
       </c>
     </row>
     <row r="776" ht="15" customHeight="1">
       <c r="A776" t="s">
+        <v>1534</v>
+      </c>
+      <c r="B776" t="s">
         <v>1535</v>
-      </c>
-      <c r="B776" t="s">
-        <v>1163</v>
       </c>
     </row>
     <row r="777" ht="15" customHeight="1">
@@ -11334,10 +11322,10 @@
       </c>
     </row>
     <row r="780" ht="15" customHeight="1">
-      <c r="A780" t="s">
+      <c r="A780" s="1" t="s">
         <v>1542</v>
       </c>
-      <c r="B780" t="s">
+      <c r="B780" s="1" t="s">
         <v>1543</v>
       </c>
     </row>
@@ -11346,23 +11334,23 @@
         <v>1544</v>
       </c>
       <c r="B781" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="782" ht="15" customHeight="1">
+      <c r="A782" t="s">
         <v>1545</v>
       </c>
-    </row>
-    <row r="782" ht="15" customHeight="1">
-      <c r="A782" s="1" t="s">
+      <c r="B782" t="s">
         <v>1546</v>
-      </c>
-      <c r="B782" s="1" t="s">
-        <v>1547</v>
       </c>
     </row>
     <row r="783" ht="15" customHeight="1">
       <c r="A783" t="s">
+        <v>1547</v>
+      </c>
+      <c r="B783" t="s">
         <v>1548</v>
-      </c>
-      <c r="B783" t="s">
-        <v>533</v>
       </c>
     </row>
     <row r="784" ht="15" customHeight="1">
@@ -11453,26 +11441,10 @@
         <v>1570</v>
       </c>
     </row>
-    <row r="795" ht="15" customHeight="1">
-      <c r="A795" t="s">
-        <v>1571</v>
-      </c>
-      <c r="B795" t="s">
-        <v>1572</v>
-      </c>
-    </row>
-    <row r="796" ht="15" customHeight="1">
-      <c r="A796" t="s">
-        <v>1573</v>
-      </c>
-      <c r="B796" t="s">
-        <v>1574</v>
-      </c>
-    </row>
   </sheetData>
   <printOptions/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>

</xml_diff>